<commit_message>
updated code other than ProductPage
</commit_message>
<xml_diff>
--- a/src/testData/eopnCartTestData.xlsx
+++ b/src/testData/eopnCartTestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\OpenCartPWFrameWorkE2E\src\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93A8AD38-3B8F-4B10-81DB-6AD77ECE6DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0E0465-C75A-41F4-AE88-CBF7E43DA1AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DDFF9CB9-96DD-44EB-954C-6729954B1980}"/>
+    <workbookView xWindow="4800" yWindow="2720" windowWidth="14400" windowHeight="7360" xr2:uid="{DDFF9CB9-96DD-44EB-954C-6729954B1980}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,15 +24,38 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>sharuBB@gmail.com</t>
+  </si>
+  <si>
+    <t>Bekind@1996</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF569CD6"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -55,8 +78,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -371,9 +397,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE7E8C7A-CE49-4CE3-80AF-6A44760EC8DD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>